<commit_message>
move "moxy_ramp" event time; update `oxcap_analysis.qmd`
</commit_message>
<xml_diff>
--- a/inst/extdata/moxy_ramp.xlsx
+++ b/inst/extdata/moxy_ramp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R-Projects\mnirs\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78CC3548-0C30-4ABC-8757-59C29C3D17A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12768D07-2A7E-4B09-B213-46225687D346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="31785" xr2:uid="{ED07EABD-9B2D-42C5-B904-3B14C8E7B28A}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="29010" windowHeight="31785" xr2:uid="{ED07EABD-9B2D-42C5-B904-3B14C8E7B28A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -34099,7 +34099,7 @@
         <v>10</v>
       </c>
       <c r="E1586">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1587" spans="1:5" x14ac:dyDescent="0.25">
@@ -34116,7 +34116,7 @@
         <v>10</v>
       </c>
       <c r="E1587">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1588" spans="1:5" x14ac:dyDescent="0.25">
@@ -34133,7 +34133,7 @@
         <v>11</v>
       </c>
       <c r="E1588">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1589" spans="1:5" x14ac:dyDescent="0.25">
@@ -34150,7 +34150,7 @@
         <v>11</v>
       </c>
       <c r="E1589">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1590" spans="1:5" x14ac:dyDescent="0.25">
@@ -34167,7 +34167,7 @@
         <v>11</v>
       </c>
       <c r="E1590">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1591" spans="1:5" x14ac:dyDescent="0.25">
@@ -34184,7 +34184,7 @@
         <v>11</v>
       </c>
       <c r="E1591">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1592" spans="1:5" x14ac:dyDescent="0.25">
@@ -34201,7 +34201,7 @@
         <v>11</v>
       </c>
       <c r="E1592">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1593" spans="1:5" x14ac:dyDescent="0.25">
@@ -34218,7 +34218,7 @@
         <v>11</v>
       </c>
       <c r="E1593">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1594" spans="1:5" x14ac:dyDescent="0.25">
@@ -34235,7 +34235,7 @@
         <v>11</v>
       </c>
       <c r="E1594">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1595" spans="1:5" x14ac:dyDescent="0.25">
@@ -34252,7 +34252,7 @@
         <v>10</v>
       </c>
       <c r="E1595">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1596" spans="1:5" x14ac:dyDescent="0.25">
@@ -34269,7 +34269,7 @@
         <v>10</v>
       </c>
       <c r="E1596">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1597" spans="1:5" x14ac:dyDescent="0.25">
@@ -34286,7 +34286,7 @@
         <v>10</v>
       </c>
       <c r="E1597">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1598" spans="1:5" x14ac:dyDescent="0.25">
@@ -34303,7 +34303,7 @@
         <v>10</v>
       </c>
       <c r="E1598">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1599" spans="1:5" x14ac:dyDescent="0.25">
@@ -34320,7 +34320,7 @@
         <v>9</v>
       </c>
       <c r="E1599">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1600" spans="1:5" x14ac:dyDescent="0.25">
@@ -34337,7 +34337,7 @@
         <v>9</v>
       </c>
       <c r="E1600">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1601" spans="1:5" x14ac:dyDescent="0.25">
@@ -34354,7 +34354,7 @@
         <v>9</v>
       </c>
       <c r="E1601">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1602" spans="1:5" x14ac:dyDescent="0.25">
@@ -34371,7 +34371,7 @@
         <v>8</v>
       </c>
       <c r="E1602">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1603" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>